<commit_message>
Compute area between curves after finding intersections
The idea behind is that the Michaelis-Menten parameters that make the most similar curve compared to the curve from the experiment have the smallest area between those curves (a perfect match would yield an area of 0).
</commit_message>
<xml_diff>
--- a/DecompositionPeroxyde.xlsx
+++ b/DecompositionPeroxyde.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Users\Administrator\source\repos\repzilon\Repzilon.Libraries\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677927C8-2C2B-4558-9815-4CC7C30BCAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A46A4A-B803-2B4A-BF92-266CB2433E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="3" xr2:uid="{B01D318F-86D7-4149-9556-C9473594BE32}"/>
+    <workbookView xWindow="42920" yWindow="-7500" windowWidth="21080" windowHeight="22380" activeTab="3" xr2:uid="{B01D318F-86D7-4149-9556-C9473594BE32}"/>
   </bookViews>
   <sheets>
     <sheet name="Michaelis-Menten lin." sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
   <si>
     <t>s</t>
   </si>
@@ -141,7 +141,43 @@
     <t>Axes</t>
   </si>
   <si>
-    <t>Michaelis-Menten</t>
+    <t>Puissance</t>
+  </si>
+  <si>
+    <t>Bas</t>
+  </si>
+  <si>
+    <t>Haut</t>
+  </si>
+  <si>
+    <t>Aire entre les courbes</t>
+  </si>
+  <si>
+    <t>MM</t>
+  </si>
+  <si>
+    <t>LB</t>
+  </si>
+  <si>
+    <t>LB(a)</t>
+  </si>
+  <si>
+    <t>EH</t>
+  </si>
+  <si>
+    <t>EH(a)</t>
+  </si>
+  <si>
+    <t>HW</t>
+  </si>
+  <si>
+    <t>DL</t>
+  </si>
+  <si>
+    <t>Aire entre</t>
+  </si>
+  <si>
+    <t>Hanes-Woolf</t>
   </si>
 </sst>
 </file>
@@ -150,9 +186,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="165" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -165,6 +201,14 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri (Corps)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -187,17 +231,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -223,7 +268,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="fr-CA"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -545,19 +590,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>3.7645116017564408E-2</c:v>
+                  <c:v>3.6519358125318382E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.9427685469272516E-2</c:v>
+                  <c:v>4.9059024807527794E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.5185165836432855E-2</c:v>
+                  <c:v>5.5399922720247283E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.1946161575092357E-2</c:v>
+                  <c:v>7.4713392391870748E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.482830944569146E-2</c:v>
+                  <c:v>9.0485957715367618E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -887,7 +932,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="fr-CA"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1367,7 +1412,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="fr-CA"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1438,7 +1483,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Hoja1!$L$2</c:f>
+              <c:f>Hoja1!$N$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1476,7 +1521,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Hoja1!$L$4:$L$5</c:f>
+              <c:f>Hoja1!$N$4:$N$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1491,7 +1536,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Hoja1!$M$4:$M$5</c:f>
+              <c:f>Hoja1!$O$4:$O$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1516,7 +1561,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Hoja1!$N$2</c:f>
+              <c:f>Hoja1!$P$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1554,7 +1599,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Hoja1!$N$4:$N$5</c:f>
+              <c:f>Hoja1!$P$4:$P$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1569,7 +1614,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Hoja1!$O$4:$O$5</c:f>
+              <c:f>Hoja1!$Q$4:$Q$5</c:f>
               <c:numCache>
                 <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1594,7 +1639,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Hoja1!$P$2</c:f>
+              <c:f>Hoja1!$R$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1632,7 +1677,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Hoja1!$P$4:$P$5</c:f>
+              <c:f>Hoja1!$R$4:$R$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1647,7 +1692,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Hoja1!$Q$4:$Q$5</c:f>
+              <c:f>Hoja1!$S$4:$S$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1672,7 +1717,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Hoja1!$R$2</c:f>
+              <c:f>Hoja1!$T$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1714,7 +1759,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Hoja1!$R$4:$R$5</c:f>
+              <c:f>Hoja1!$T$4:$T$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1729,7 +1774,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Hoja1!$S$4:$S$5</c:f>
+              <c:f>Hoja1!$U$4:$U$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1754,7 +1799,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Hoja1!$T$2</c:f>
+              <c:f>Hoja1!$V$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1796,7 +1841,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Hoja1!$T$4:$T$5</c:f>
+              <c:f>Hoja1!$V$4:$V$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1811,7 +1856,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Hoja1!$U$4:$U$5</c:f>
+              <c:f>Hoja1!$W$4:$W$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1915,7 +1960,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="fr-CA"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3809,7 +3854,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8672180" cy="6302006"/>
+    <xdr:ext cx="8676033" cy="6294783"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Gráfico 1">
@@ -3842,7 +3887,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8659091" cy="6285057"/>
+    <xdr:ext cx="8676033" cy="6294783"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Graphique 1">
@@ -3875,7 +3920,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8659091" cy="6285057"/>
+    <xdr:ext cx="8676033" cy="6294783"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Graphique 1">
@@ -4201,29 +4246,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B5621EF-2F33-5D4E-AA64-015F90897498}">
-  <dimension ref="A1:U6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <dimension ref="A1:W30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="3.875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="3.875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="6.125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="4.875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.1640625" customWidth="1"/>
+    <col min="9" max="9" width="13" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="3.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="3.83203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.83203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="6.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="19.5">
+    <row r="1" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4239,29 +4285,29 @@
       <c r="E1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>12.5</v>
       </c>
@@ -4273,52 +4319,52 @@
         <v>3.6999999999999998E-2</v>
       </c>
       <c r="D2">
-        <f>$I$2*LOG10(A2)+$I$3</f>
+        <f>$K$2*LOG10(A2)+$K$3</f>
         <v>3.7284943247737408E-2</v>
       </c>
       <c r="E2">
-        <f>($I$4*A2)/($I$5+A2)</f>
-        <v>3.7645116017564408E-2</v>
-      </c>
-      <c r="G2" s="3" t="s">
+        <f>($K$4*A2)/($K$5+A2)</f>
+        <v>3.6519358125318382E-2</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>1</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>5.9481399999999997E-2</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>0</v>
       </c>
-      <c r="L2" s="2">
+      <c r="N2" s="5">
         <f>A2</f>
         <v>12.5</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2">
+      <c r="O2" s="5"/>
+      <c r="P2" s="5">
         <f>A3</f>
         <v>20</v>
       </c>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2">
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5">
         <f>A4</f>
         <v>25</v>
       </c>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2">
+      <c r="S2" s="5"/>
+      <c r="T2" s="5">
         <f>A5</f>
         <v>50</v>
       </c>
-      <c r="S2" s="2"/>
-      <c r="T2" s="2">
+      <c r="U2" s="5"/>
+      <c r="V2" s="5">
         <f>A6</f>
         <v>100</v>
       </c>
-      <c r="U2" s="2"/>
+      <c r="W2" s="5"/>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>20</v>
       </c>
@@ -4330,28 +4376,22 @@
         <v>0.05</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D6" si="1">$I$2*LOG10(A3)+$I$3</f>
+        <f t="shared" ref="D3:D6" si="1">$K$2*LOG10(A3)+$K$3</f>
         <v>4.9426285584087536E-2</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E6" si="2">($I$4*A3)/($I$5+A3)</f>
-        <v>4.9427685469272516E-2</v>
-      </c>
-      <c r="G3" s="3"/>
-      <c r="H3" t="s">
+        <f t="shared" ref="E3:E6" si="2">($K$4*A3)/($K$5+A3)</f>
+        <v>4.9059024807527794E-2</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" t="s">
         <v>2</v>
       </c>
-      <c r="I3">
+      <c r="K3">
         <v>-2.7960800000000001E-2</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>18</v>
-      </c>
-      <c r="L3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M3" t="s">
-        <v>14</v>
       </c>
       <c r="N3" t="s">
         <v>13</v>
@@ -4377,8 +4417,14 @@
       <c r="U3" t="s">
         <v>14</v>
       </c>
+      <c r="V3" t="s">
+        <v>13</v>
+      </c>
+      <c r="W3" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="4" spans="1:21" ht="19.5">
+    <row r="4" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>25</v>
       </c>
@@ -4395,58 +4441,57 @@
       </c>
       <c r="E4">
         <f t="shared" si="2"/>
-        <v>5.5185165836432855E-2</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" t="s">
+        <v>5.5399922720247283E-2</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="4">
-        <f>I2*4/LN(10)</f>
-        <v>0.10332977518352032</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="K4" s="2">
+        <v>0.1147</v>
+      </c>
+      <c r="M4" t="s">
         <v>17</v>
-      </c>
-      <c r="L4">
-        <f>-1*L2</f>
-        <v>-12.5</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
       </c>
       <c r="N4">
         <f>-1*N2</f>
-        <v>-20</v>
+        <v>-12.5</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
         <f>-1*P2</f>
-        <v>-25</v>
+        <v>-20</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
       <c r="R4">
         <f>-1*R2</f>
-        <v>-50</v>
+        <v>-25</v>
       </c>
       <c r="S4">
         <v>0</v>
       </c>
       <c r="T4">
         <f>-1*T2</f>
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="U4">
         <v>0</v>
       </c>
+      <c r="V4">
+        <f>-1*V2</f>
+        <v>-100</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:21" ht="19.5">
+    <row r="5" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>50</v>
       </c>
@@ -4463,56 +4508,55 @@
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>7.1946161575092357E-2</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" t="s">
+        <v>7.4713392391870748E-2</v>
+      </c>
+      <c r="I5" s="4"/>
+      <c r="J5" t="s">
         <v>5</v>
       </c>
-      <c r="I5" s="5">
-        <f>10^((0.5*I4-I3)/I2)</f>
-        <v>21.810485035863902</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="K5" s="3">
+        <v>26.76</v>
+      </c>
+      <c r="M5" t="s">
         <v>16</v>
       </c>
-      <c r="L5">
+      <c r="N5">
         <v>0</v>
       </c>
-      <c r="M5">
+      <c r="O5">
         <f>C2</f>
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="N5">
+      <c r="P5">
         <v>0</v>
       </c>
-      <c r="O5" s="1">
+      <c r="Q5" s="1">
         <f>C3</f>
         <v>0.05</v>
       </c>
-      <c r="P5">
+      <c r="R5">
         <v>0</v>
       </c>
-      <c r="Q5">
+      <c r="S5">
         <f>C4</f>
         <v>5.5E-2</v>
       </c>
-      <c r="R5">
+      <c r="T5">
         <v>0</v>
       </c>
-      <c r="S5">
+      <c r="U5">
         <f>C5</f>
         <v>7.2999999999999995E-2</v>
       </c>
-      <c r="T5">
+      <c r="V5">
         <v>0</v>
       </c>
-      <c r="U5">
+      <c r="W5">
         <f>C6</f>
         <v>9.0999999999999998E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>100</v>
       </c>
@@ -4529,20 +4573,1032 @@
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>8.482830944569146E-2</v>
-      </c>
+        <v>9.0485957715367618E-2</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" t="s">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>1.3624600000000001E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="I7" s="4"/>
+      <c r="J7" t="s">
+        <v>2</v>
+      </c>
+      <c r="K7">
+        <v>0.42139300000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+    </row>
+    <row r="10" spans="1:23" ht="18" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="4">
+        <v>0.1033</v>
+      </c>
+      <c r="C11" s="4">
+        <v>21.81</v>
+      </c>
+      <c r="D11" s="6">
+        <v>12.5</v>
+      </c>
+      <c r="E11">
+        <v>21.8105098199681</v>
+      </c>
+      <c r="F11">
+        <f>D11*($K$2/LN(10)*LN(D11)-($K$2/LN(10))+$K$3)</f>
+        <v>0.14315624314821659</v>
+      </c>
+      <c r="G11">
+        <f>E11*($K$2/LN(10)*LN(E11)-($K$2/LN(10))+$K$3)</f>
+        <v>0.56341940931815915</v>
+      </c>
+      <c r="H11">
+        <f>G11-F11</f>
+        <v>0.42026316616994253</v>
+      </c>
+      <c r="I11">
+        <f>$B$11*(D11-$C$11*LN(ABS(D11+$C$11)))</f>
+        <v>-6.673993781733782</v>
+      </c>
+      <c r="J11">
+        <f>$B$11*(E11-$C$11*LN(ABS(E11+$C$11)))</f>
+        <v>-6.253135737741883</v>
+      </c>
+      <c r="K11">
+        <f>J11-I11</f>
+        <v>0.42085804399189897</v>
+      </c>
+      <c r="L11">
+        <f>ABS(H11-K11)</f>
+        <v>5.9487782195644101E-4</v>
+      </c>
+      <c r="M11" s="4">
+        <f>SUM(L11:L12)</f>
+        <v>0.19081359290049127</v>
+      </c>
+      <c r="N11" s="4"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12">
+        <f>E11</f>
+        <v>21.8105098199681</v>
+      </c>
+      <c r="E12" s="6">
+        <v>100</v>
+      </c>
+      <c r="F12">
+        <f>D12*($K$2/LN(10)*LN(D12)-($K$2/LN(10))+$K$3)</f>
+        <v>0.56341940931815915</v>
+      </c>
+      <c r="G12">
+        <f>E12*($K$2/LN(10)*LN(E12)-($K$2/LN(10))+$K$3)</f>
+        <v>6.5169556204119905</v>
+      </c>
+      <c r="H12">
+        <f>G12-F12</f>
+        <v>5.953536211093831</v>
+      </c>
+      <c r="I12">
+        <f>$B$11*(D12-$C$11*LN(ABS(D12+$C$11)))</f>
+        <v>-6.253135737741883</v>
+      </c>
+      <c r="J12">
+        <f>$B$11*(E12-$C$11*LN(ABS(E12+$C$11)))</f>
+        <v>-0.48981824172658694</v>
+      </c>
+      <c r="K12">
+        <f>J12-I12</f>
+        <v>5.7633174960152962</v>
+      </c>
+      <c r="L12">
+        <f>ABS(H12-K12)</f>
+        <v>0.19021871507853483</v>
+      </c>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="4">
+        <v>0.1118</v>
+      </c>
+      <c r="C13" s="4">
+        <v>25.24</v>
+      </c>
+      <c r="D13">
+        <f>$D$11</f>
+        <v>12.5</v>
+      </c>
+      <c r="E13">
+        <v>20.147617441101598</v>
+      </c>
+      <c r="F13">
+        <f t="shared" ref="F13:F15" si="3">D13*($K$2/LN(10)*LN(D13)-($K$2/LN(10))+$K$3)</f>
+        <v>0.14315624314821659</v>
+      </c>
+      <c r="G13">
+        <f t="shared" ref="G13:G15" si="4">E13*($K$2/LN(10)*LN(E13)-($K$2/LN(10))+$K$3)</f>
+        <v>0.47918705587998178</v>
+      </c>
+      <c r="H13">
+        <f t="shared" ref="H13:H15" si="5">G13-F13</f>
+        <v>0.33603081273176516</v>
+      </c>
+      <c r="I13">
+        <f>$B$13*(D13-$C$13*LN(ABS(D13+$C$13)))</f>
+        <v>-8.8477834026611095</v>
+      </c>
+      <c r="J13">
+        <f>$B$13*(E13-$C$13*LN(ABS(E13+$C$13)))</f>
+        <v>-8.5134607829342563</v>
+      </c>
+      <c r="K13">
+        <f>J13-I13</f>
+        <v>0.33432261972685318</v>
+      </c>
+      <c r="L13">
+        <f>ABS(H13-K13)</f>
+        <v>1.7081930049119842E-3</v>
+      </c>
+      <c r="M13" s="4">
+        <f>SUM(L13:L15)</f>
+        <v>6.7239401917722597E-2</v>
+      </c>
+      <c r="N13" s="4"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14">
+        <f>E13</f>
+        <v>20.147617441101598</v>
+      </c>
+      <c r="E14">
+        <v>75.907855428222305</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="3"/>
+        <v>0.47918705587998178</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="4"/>
+        <v>4.4063631683266218</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="5"/>
+        <v>3.9271761124466398</v>
+      </c>
+      <c r="I14">
+        <f t="shared" ref="I14:J15" si="6">$B$13*(D14-$C$13*LN(ABS(D14+$C$13)))</f>
+        <v>-8.5134607829342563</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="6"/>
+        <v>-4.5407244232533115</v>
+      </c>
+      <c r="K14">
+        <f t="shared" ref="K14:K15" si="7">J14-I14</f>
+        <v>3.9727363596809449</v>
+      </c>
+      <c r="L14">
+        <f t="shared" ref="L14:L15" si="8">ABS(H14-K14)</f>
+        <v>4.5560247234305074E-2</v>
+      </c>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15">
+        <f>E14</f>
+        <v>75.907855428222305</v>
+      </c>
+      <c r="E15">
+        <v>100</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="3"/>
+        <v>4.4063631683266218</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="4"/>
+        <v>6.5169556204119905</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="5"/>
+        <v>2.1105924520853687</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="6"/>
+        <v>-4.5407244232533115</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="6"/>
+        <v>-2.4501029328464483</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="7"/>
+        <v>2.0906214904068632</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="8"/>
+        <v>1.9970961678505539E-2</v>
+      </c>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="4">
+        <v>0.1115</v>
+      </c>
+      <c r="C16" s="4">
+        <v>25.13</v>
+      </c>
+      <c r="D16">
+        <f>$D$11</f>
+        <v>12.5</v>
+      </c>
+      <c r="E16">
+        <v>20.033836517991499</v>
+      </c>
+      <c r="F16">
+        <f t="shared" ref="F16:F30" si="9">D16*($K$2/LN(10)*LN(D16)-($K$2/LN(10))+$K$3)</f>
+        <v>0.14315624314821659</v>
+      </c>
+      <c r="G16">
+        <f t="shared" ref="G16:G30" si="10">E16*($K$2/LN(10)*LN(E16)-($K$2/LN(10))+$K$3)</f>
+        <v>0.47354998814449217</v>
+      </c>
+      <c r="H16">
+        <f t="shared" ref="H16:H30" si="11">G16-F16</f>
+        <v>0.33039374499627561</v>
+      </c>
+      <c r="I16">
+        <f>$B$16*(D16-$C$16*LN(ABS(D16+$C$16)))</f>
+        <v>-8.7713319570961552</v>
+      </c>
+      <c r="J16">
+        <f>$B$16*(E16-$C$16*LN(ABS(E16+$C$16)))</f>
+        <v>-8.4426595009360579</v>
+      </c>
+      <c r="K16">
+        <f t="shared" ref="K16:K18" si="12">J16-I16</f>
+        <v>0.32867245616009733</v>
+      </c>
+      <c r="L16">
+        <f t="shared" ref="L16:L18" si="13">ABS(H16-K16)</f>
+        <v>1.7212888361782808E-3</v>
+      </c>
+      <c r="M16" s="4">
+        <f>SUM(L16:L18)</f>
+        <v>6.6438104392574249E-2</v>
+      </c>
+      <c r="N16" s="4"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17">
+        <f>E16</f>
+        <v>20.033836517991499</v>
+      </c>
+      <c r="E17">
+        <v>74.442933006459498</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="9"/>
+        <v>0.47354998814449217</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="10"/>
+        <v>4.283851118395301</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="11"/>
+        <v>3.8103011302508087</v>
+      </c>
+      <c r="I17">
+        <f t="shared" ref="I17:J18" si="14">$B$16*(D17-$C$16*LN(ABS(D17+$C$16)))</f>
+        <v>-8.4426595009360579</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="14"/>
+        <v>-4.5912847840144053</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="12"/>
+        <v>3.8513747169216526</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="13"/>
+        <v>4.107358667084382E-2</v>
+      </c>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18">
+        <f>E17</f>
+        <v>74.442933006459498</v>
+      </c>
+      <c r="E18">
+        <v>100</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="9"/>
+        <v>4.283851118395301</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="10"/>
+        <v>6.5169556204119905</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="11"/>
+        <v>2.2331045020166895</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="14"/>
+        <v>-4.5912847840144053</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="14"/>
+        <v>-2.3818235108832679</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="12"/>
+        <v>2.2094612731311374</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="13"/>
+        <v>2.3643228885552148E-2</v>
+      </c>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="4">
+        <v>0.11260000000000001</v>
+      </c>
+      <c r="C19" s="4">
+        <v>25.61</v>
+      </c>
+      <c r="D19">
+        <f>$D$11</f>
+        <v>12.5</v>
+      </c>
+      <c r="E19">
+        <v>20.6619897321903</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="9"/>
+        <v>0.14315624314821659</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="10"/>
+        <v>0.50487647151218762</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="11"/>
+        <v>0.361720228363971</v>
+      </c>
+      <c r="I19">
+        <f>$B$19*(D19-$C$19*LN(ABS(D19+$C$19)))</f>
+        <v>-9.0904917360420843</v>
+      </c>
+      <c r="J19">
+        <f>$B$19*(E19-$C$19*LN(ABS(E19+$C$19)))</f>
+        <v>-8.731060056166438</v>
+      </c>
+      <c r="K19">
+        <f t="shared" ref="K19:K21" si="15">J19-I19</f>
+        <v>0.35943167987564628</v>
+      </c>
+      <c r="L19">
+        <f t="shared" ref="L19:L21" si="16">ABS(H19-K19)</f>
+        <v>2.2885484883247154E-3</v>
+      </c>
+      <c r="M19" s="4">
+        <f>SUM(L19:L21)</f>
+        <v>6.9241854143262338E-2</v>
+      </c>
+      <c r="N19" s="4"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20">
+        <f>E19</f>
+        <v>20.6619897321903</v>
+      </c>
+      <c r="E20">
+        <v>80.604418907483605</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="9"/>
+        <v>0.50487647151218762</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="10"/>
+        <v>4.8039951221831991</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="11"/>
+        <v>4.2991186506710113</v>
+      </c>
+      <c r="I20">
+        <f t="shared" ref="I20:J21" si="17">$B$19*(D20-$C$19*LN(ABS(D20+$C$19)))</f>
+        <v>-8.731060056166438</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="17"/>
+        <v>-4.3776637441454449</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="15"/>
+        <v>4.3533963120209931</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="16"/>
+        <v>5.4277661349981798E-2</v>
+      </c>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21">
+        <f>E20</f>
+        <v>80.604418907483605</v>
+      </c>
+      <c r="E21">
+        <v>100</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="9"/>
+        <v>4.8039951221831991</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="10"/>
+        <v>6.5169556204119905</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="11"/>
+        <v>1.7129604982287914</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="17"/>
+        <v>-4.3776637441454449</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="17"/>
+        <v>-2.6773788902216094</v>
+      </c>
+      <c r="K21">
+        <f t="shared" si="15"/>
+        <v>1.7002848539238355</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="16"/>
+        <v>1.2675644304955824E-2</v>
+      </c>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="4">
+        <v>0.11269999999999999</v>
+      </c>
+      <c r="C22" s="4">
+        <v>25.47</v>
+      </c>
+      <c r="D22">
+        <f>$D$11</f>
+        <v>12.5</v>
+      </c>
+      <c r="E22">
+        <v>18.437861846839699</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="9"/>
+        <v>0.14315624314821659</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="10"/>
+        <v>0.39628481903313884</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="11"/>
+        <v>0.25312857588492221</v>
+      </c>
+      <c r="I22">
+        <f>$B$22*(D22-$C$22*LN(ABS(D22+$C$22)))</f>
+        <v>-9.0305612515789697</v>
+      </c>
+      <c r="J22">
+        <f>$B$22*(E22-$C$22*LN(ABS(E22+$C$22)))</f>
+        <v>-8.7784347992292702</v>
+      </c>
+      <c r="K22">
+        <f t="shared" ref="K22:K24" si="18">J22-I22</f>
+        <v>0.25212645234969955</v>
+      </c>
+      <c r="L22">
+        <f t="shared" ref="L22:L24" si="19">ABS(H22-K22)</f>
+        <v>1.0021235352226654E-3</v>
+      </c>
+      <c r="M22" s="4">
+        <f>SUM(L22:L24)</f>
+        <v>7.7324198207290529E-2</v>
+      </c>
+      <c r="N22" s="4"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23">
+        <f>E22</f>
+        <v>18.437861846839699</v>
+      </c>
+      <c r="E23">
+        <v>83.712210015958405</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="9"/>
+        <v>0.39628481903313884</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="10"/>
+        <v>5.0710283832474241</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="11"/>
+        <v>4.6747435642142854</v>
+      </c>
+      <c r="I23">
+        <f t="shared" ref="I23:J24" si="20">$B$22*(D23-$C$22*LN(ABS(D23+$C$22)))</f>
+        <v>-8.7784347992292702</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="20"/>
+        <v>-4.0367970130479067</v>
+      </c>
+      <c r="K23">
+        <f t="shared" si="18"/>
+        <v>4.7416377861813634</v>
+      </c>
+      <c r="L23">
+        <f t="shared" si="19"/>
+        <v>6.689422196707806E-2</v>
+      </c>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24">
+        <f>E23</f>
+        <v>83.712210015958405</v>
+      </c>
+      <c r="E24">
+        <v>100</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="9"/>
+        <v>5.0710283832474241</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="10"/>
+        <v>6.5169556204119905</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="11"/>
+        <v>1.4459272371645664</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="20"/>
+        <v>-4.0367970130479067</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="20"/>
+        <v>-2.6002976285883301</v>
+      </c>
+      <c r="K24">
+        <f t="shared" si="18"/>
+        <v>1.4364993844595766</v>
+      </c>
+      <c r="L24">
+        <f t="shared" si="19"/>
+        <v>9.4278527049898031E-3</v>
+      </c>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="4">
+        <v>0.1147</v>
+      </c>
+      <c r="C25" s="4">
+        <v>26.76</v>
+      </c>
+      <c r="D25">
+        <f>$D$11</f>
+        <v>12.5</v>
+      </c>
+      <c r="E25">
+        <v>23.274788136571999</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="9"/>
+        <v>0.14315624314821659</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="10"/>
+        <v>0.6403134748816397</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="11"/>
+        <v>0.49715723173342308</v>
+      </c>
+      <c r="I25">
+        <f>$B$25*(D25-$C$25*LN(ABS(D25+$C$25)))</f>
+        <v>-9.8314781102777307</v>
+      </c>
+      <c r="J25">
+        <f>$B$25*(E25-$C$25*LN(ABS(E25+$C$25)))</f>
+        <v>-9.339970489023468</v>
+      </c>
+      <c r="K25">
+        <f t="shared" ref="K25:K27" si="21">J25-I25</f>
+        <v>0.49150762125426262</v>
+      </c>
+      <c r="L25">
+        <f t="shared" ref="L25:L27" si="22">ABS(H25-K25)</f>
+        <v>5.6496104791604607E-3</v>
+      </c>
+      <c r="M25" s="4">
+        <f>SUM(L25:L27)</f>
+        <v>8.0197419964009753E-2</v>
+      </c>
+      <c r="N25" s="4"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26">
+        <f>E25</f>
+        <v>23.274788136571999</v>
+      </c>
+      <c r="E26">
+        <v>91.828309176174798</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="9"/>
+        <v>0.6403134748816397</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="10"/>
+        <v>5.7821854502295738</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="11"/>
+        <v>5.1418719753479341</v>
+      </c>
+      <c r="I26">
+        <f t="shared" ref="I26:J27" si="23">$B$25*(D26-$C$25*LN(ABS(D26+$C$25)))</f>
+        <v>-9.339970489023468</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="23"/>
+        <v>-4.1255636023414919</v>
+      </c>
+      <c r="K26">
+        <f t="shared" si="21"/>
+        <v>5.2144068866819762</v>
+      </c>
+      <c r="L26">
+        <f t="shared" si="22"/>
+        <v>7.2534911334042107E-2</v>
+      </c>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27">
+        <f>E26</f>
+        <v>91.828309176174798</v>
+      </c>
+      <c r="E27">
+        <v>100</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="9"/>
+        <v>5.7821854502295738</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="10"/>
+        <v>6.5169556204119905</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="11"/>
+        <v>0.73477017018241675</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="23"/>
+        <v>-4.1255636023414919</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="23"/>
+        <v>-3.3928063303098823</v>
+      </c>
+      <c r="K27">
+        <f t="shared" si="21"/>
+        <v>0.73275727203160956</v>
+      </c>
+      <c r="L27">
+        <f t="shared" si="22"/>
+        <v>2.0128981508071853E-3</v>
+      </c>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="4">
+        <v>0.1115</v>
+      </c>
+      <c r="C28" s="4">
+        <v>25.06</v>
+      </c>
+      <c r="D28">
+        <f>$D$11</f>
+        <v>12.5</v>
+      </c>
+      <c r="E28">
+        <v>19.2292181061114</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="9"/>
+        <v>0.14315624314821659</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="10"/>
+        <v>0.43416865529613313</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="11"/>
+        <v>0.29101241214791651</v>
+      </c>
+      <c r="I28">
+        <f>$B$28*(D28-$C$28*LN(ABS(D28+$C$28)))</f>
+        <v>-8.7378143227604586</v>
+      </c>
+      <c r="J28">
+        <f>$B$28*(E28-$C$28*LN(ABS(E28+$C$28)))</f>
+        <v>-8.4479935131197408</v>
+      </c>
+      <c r="K28">
+        <f t="shared" ref="K28:K30" si="24">J28-I28</f>
+        <v>0.28982080964071777</v>
+      </c>
+      <c r="L28">
+        <f t="shared" ref="L28:L30" si="25">ABS(H28-K28)</f>
+        <v>1.1916025071987413E-3</v>
+      </c>
+      <c r="M28" s="4">
+        <f>SUM(L28:L30)</f>
+        <v>6.8379533125184633E-2</v>
+      </c>
+      <c r="N28" s="4"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29">
+        <f>E28</f>
+        <v>19.2292181061114</v>
+      </c>
+      <c r="E29">
+        <v>75.007571946818402</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="9"/>
+        <v>0.43416865529613313</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="10"/>
+        <v>4.3309846937527059</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="11"/>
+        <v>3.8968160384565729</v>
+      </c>
+      <c r="I29">
+        <f t="shared" ref="I29:J30" si="26">$B$28*(D29-$C$28*LN(ABS(D29+$C$28)))</f>
+        <v>-8.4479935131197408</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="26"/>
+        <v>-4.5062636608747315</v>
+      </c>
+      <c r="K29">
+        <f t="shared" si="24"/>
+        <v>3.9417298522450093</v>
+      </c>
+      <c r="L29">
+        <f t="shared" si="25"/>
+        <v>4.4913813788436396E-2</v>
+      </c>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30">
+        <f>E29</f>
+        <v>75.007571946818402</v>
+      </c>
+      <c r="E30">
+        <v>100</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="9"/>
+        <v>4.3309846937527059</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="10"/>
+        <v>6.5169556204119905</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="11"/>
+        <v>2.1859709266592846</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="26"/>
+        <v>-4.5062636608747315</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="26"/>
+        <v>-2.3425668510449964</v>
+      </c>
+      <c r="K30">
+        <f t="shared" si="24"/>
+        <v>2.1636968098297351</v>
+      </c>
+      <c r="L30">
+        <f t="shared" si="25"/>
+        <v>2.2274116829549495E-2</v>
+      </c>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="L1:U1"/>
-    <mergeCell ref="R2:S2"/>
+  <mergeCells count="41">
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="N1:W1"/>
     <mergeCell ref="T2:U2"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="I4:I5"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="A9:N9"/>
+    <mergeCell ref="M16:N18"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="M19:N21"/>
+    <mergeCell ref="M22:N24"/>
+    <mergeCell ref="M25:N27"/>
+    <mergeCell ref="M28:N30"/>
+    <mergeCell ref="M11:N12"/>
+    <mergeCell ref="M13:N15"/>
   </mergeCells>
+  <conditionalFormatting sqref="M11:N30">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Promoted optimal Michaelis-Menten parameters to the library
</commit_message>
<xml_diff>
--- a/DecompositionPeroxyde.xlsx
+++ b/DecompositionPeroxyde.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrener/Projects/Repzilon.Libraries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A46A4A-B803-2B4A-BF92-266CB2433E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8A84D5-DBE2-F944-8C7E-7C3AAE303997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42920" yWindow="-7500" windowWidth="21080" windowHeight="22380" activeTab="3" xr2:uid="{B01D318F-86D7-4149-9556-C9473594BE32}"/>
+    <workbookView xWindow="25600" yWindow="-7500" windowWidth="38400" windowHeight="23500" xr2:uid="{B01D318F-86D7-4149-9556-C9473594BE32}"/>
   </bookViews>
   <sheets>
     <sheet name="Michaelis-Menten lin." sheetId="2" r:id="rId1"/>
@@ -236,13 +236,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -590,19 +590,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>3.6519358125318382E-2</c:v>
+                  <c:v>3.7038267339888395E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.9059024807527794E-2</c:v>
+                  <c:v>4.9412807445158434E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.5399922720247283E-2</c:v>
+                  <c:v>5.5605425892679042E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.4713392391870748E-2</c:v>
+                  <c:v>7.4204711832823109E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>9.0485957715367618E-2</c:v>
+                  <c:v>8.9107328378486381E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4294,18 +4294,18 @@
       <c r="K1" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-      <c r="U1" s="5"/>
-      <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="6"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2">
@@ -4324,9 +4324,9 @@
       </c>
       <c r="E2">
         <f>($K$4*A2)/($K$5+A2)</f>
-        <v>3.6519358125318382E-2</v>
-      </c>
-      <c r="I2" s="4" t="s">
+        <v>3.7038267339888395E-2</v>
+      </c>
+      <c r="I2" s="5" t="s">
         <v>11</v>
       </c>
       <c r="J2" t="s">
@@ -4338,31 +4338,31 @@
       <c r="M2" t="s">
         <v>0</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="6">
         <f>A2</f>
         <v>12.5</v>
       </c>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5">
+      <c r="O2" s="6"/>
+      <c r="P2" s="6">
         <f>A3</f>
         <v>20</v>
       </c>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="5">
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6">
         <f>A4</f>
         <v>25</v>
       </c>
-      <c r="S2" s="5"/>
-      <c r="T2" s="5">
+      <c r="S2" s="6"/>
+      <c r="T2" s="6">
         <f>A5</f>
         <v>50</v>
       </c>
-      <c r="U2" s="5"/>
-      <c r="V2" s="5">
+      <c r="U2" s="6"/>
+      <c r="V2" s="6">
         <f>A6</f>
         <v>100</v>
       </c>
-      <c r="W2" s="5"/>
+      <c r="W2" s="6"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3">
@@ -4381,9 +4381,9 @@
       </c>
       <c r="E3">
         <f t="shared" ref="E3:E6" si="2">($K$4*A3)/($K$5+A3)</f>
-        <v>4.9059024807527794E-2</v>
-      </c>
-      <c r="I3" s="4"/>
+        <v>4.9412807445158434E-2</v>
+      </c>
+      <c r="I3" s="5"/>
       <c r="J3" t="s">
         <v>2</v>
       </c>
@@ -4441,16 +4441,16 @@
       </c>
       <c r="E4">
         <f t="shared" si="2"/>
-        <v>5.5399922720247283E-2</v>
-      </c>
-      <c r="I4" s="4" t="s">
+        <v>5.5605425892679042E-2</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>31</v>
       </c>
       <c r="J4" t="s">
         <v>4</v>
       </c>
       <c r="K4" s="2">
-        <v>0.1147</v>
+        <v>0.1115</v>
       </c>
       <c r="M4" t="s">
         <v>17</v>
@@ -4508,14 +4508,14 @@
       </c>
       <c r="E5">
         <f t="shared" si="2"/>
-        <v>7.4713392391870748E-2</v>
-      </c>
-      <c r="I5" s="4"/>
+        <v>7.4204711832823109E-2</v>
+      </c>
+      <c r="I5" s="5"/>
       <c r="J5" t="s">
         <v>5</v>
       </c>
       <c r="K5" s="3">
-        <v>26.76</v>
+        <v>25.13</v>
       </c>
       <c r="M5" t="s">
         <v>16</v>
@@ -4573,9 +4573,9 @@
       </c>
       <c r="E6">
         <f t="shared" si="2"/>
-        <v>9.0485957715367618E-2</v>
-      </c>
-      <c r="I6" s="4" t="s">
+        <v>8.9107328378486381E-2</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>19</v>
       </c>
       <c r="J6" t="s">
@@ -4586,7 +4586,7 @@
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="I7" s="4"/>
+      <c r="I7" s="5"/>
       <c r="J7" t="s">
         <v>2</v>
       </c>
@@ -4595,22 +4595,22 @@
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
     </row>
     <row r="10" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
@@ -4625,33 +4625,33 @@
       <c r="E10" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5" t="s">
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5" t="s">
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="5">
         <v>0.1033</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="5">
         <v>21.81</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <v>12.5</v>
       </c>
       <c r="E11">
@@ -4685,21 +4685,21 @@
         <f>ABS(H11-K11)</f>
         <v>5.9487782195644101E-4</v>
       </c>
-      <c r="M11" s="4">
+      <c r="M11" s="5">
         <f>SUM(L11:L12)</f>
         <v>0.19081359290049127</v>
       </c>
-      <c r="N11" s="4"/>
+      <c r="N11" s="5"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
       <c r="D12">
         <f>E11</f>
         <v>21.8105098199681</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="4">
         <v>100</v>
       </c>
       <c r="F12">
@@ -4730,17 +4730,17 @@
         <f>ABS(H12-K12)</f>
         <v>0.19021871507853483</v>
       </c>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="5">
         <v>0.1118</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="5">
         <v>25.24</v>
       </c>
       <c r="D13">
@@ -4778,16 +4778,16 @@
         <f>ABS(H13-K13)</f>
         <v>1.7081930049119842E-3</v>
       </c>
-      <c r="M13" s="4">
+      <c r="M13" s="5">
         <f>SUM(L13:L15)</f>
         <v>6.7239401917722597E-2</v>
       </c>
-      <c r="N13" s="4"/>
+      <c r="N13" s="5"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
       <c r="D14">
         <f>E13</f>
         <v>20.147617441101598</v>
@@ -4823,13 +4823,13 @@
         <f t="shared" ref="L14:L15" si="8">ABS(H14-K14)</f>
         <v>4.5560247234305074E-2</v>
       </c>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
       <c r="D15">
         <f>E14</f>
         <v>75.907855428222305</v>
@@ -4865,17 +4865,17 @@
         <f t="shared" si="8"/>
         <v>1.9970961678505539E-2</v>
       </c>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="5">
         <v>0.1115</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="5">
         <v>25.13</v>
       </c>
       <c r="D16">
@@ -4913,16 +4913,16 @@
         <f t="shared" ref="L16:L18" si="13">ABS(H16-K16)</f>
         <v>1.7212888361782808E-3</v>
       </c>
-      <c r="M16" s="4">
+      <c r="M16" s="5">
         <f>SUM(L16:L18)</f>
         <v>6.6438104392574249E-2</v>
       </c>
-      <c r="N16" s="4"/>
+      <c r="N16" s="5"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
       <c r="D17">
         <f>E16</f>
         <v>20.033836517991499</v>
@@ -4958,13 +4958,13 @@
         <f t="shared" si="13"/>
         <v>4.107358667084382E-2</v>
       </c>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
       <c r="D18">
         <f>E17</f>
         <v>74.442933006459498</v>
@@ -5000,17 +5000,17 @@
         <f t="shared" si="13"/>
         <v>2.3643228885552148E-2</v>
       </c>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="5">
         <v>0.11260000000000001</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="5">
         <v>25.61</v>
       </c>
       <c r="D19">
@@ -5048,16 +5048,16 @@
         <f t="shared" ref="L19:L21" si="16">ABS(H19-K19)</f>
         <v>2.2885484883247154E-3</v>
       </c>
-      <c r="M19" s="4">
+      <c r="M19" s="5">
         <f>SUM(L19:L21)</f>
         <v>6.9241854143262338E-2</v>
       </c>
-      <c r="N19" s="4"/>
+      <c r="N19" s="5"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
       <c r="D20">
         <f>E19</f>
         <v>20.6619897321903</v>
@@ -5093,13 +5093,13 @@
         <f t="shared" si="16"/>
         <v>5.4277661349981798E-2</v>
       </c>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
       <c r="D21">
         <f>E20</f>
         <v>80.604418907483605</v>
@@ -5135,17 +5135,17 @@
         <f t="shared" si="16"/>
         <v>1.2675644304955824E-2</v>
       </c>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="5">
         <v>0.11269999999999999</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="5">
         <v>25.47</v>
       </c>
       <c r="D22">
@@ -5183,16 +5183,16 @@
         <f t="shared" ref="L22:L24" si="19">ABS(H22-K22)</f>
         <v>1.0021235352226654E-3</v>
       </c>
-      <c r="M22" s="4">
+      <c r="M22" s="5">
         <f>SUM(L22:L24)</f>
         <v>7.7324198207290529E-2</v>
       </c>
-      <c r="N22" s="4"/>
+      <c r="N22" s="5"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
       <c r="D23">
         <f>E22</f>
         <v>18.437861846839699</v>
@@ -5228,13 +5228,13 @@
         <f t="shared" si="19"/>
         <v>6.689422196707806E-2</v>
       </c>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="5"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
       <c r="D24">
         <f>E23</f>
         <v>83.712210015958405</v>
@@ -5270,17 +5270,17 @@
         <f t="shared" si="19"/>
         <v>9.4278527049898031E-3</v>
       </c>
-      <c r="M24" s="4"/>
-      <c r="N24" s="4"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="5">
         <v>0.1147</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="5">
         <v>26.76</v>
       </c>
       <c r="D25">
@@ -5318,16 +5318,16 @@
         <f t="shared" ref="L25:L27" si="22">ABS(H25-K25)</f>
         <v>5.6496104791604607E-3</v>
       </c>
-      <c r="M25" s="4">
+      <c r="M25" s="5">
         <f>SUM(L25:L27)</f>
         <v>8.0197419964009753E-2</v>
       </c>
-      <c r="N25" s="4"/>
+      <c r="N25" s="5"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
       <c r="D26">
         <f>E25</f>
         <v>23.274788136571999</v>
@@ -5363,13 +5363,13 @@
         <f t="shared" si="22"/>
         <v>7.2534911334042107E-2</v>
       </c>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
+      <c r="M26" s="5"/>
+      <c r="N26" s="5"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
+      <c r="A27" s="5"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
       <c r="D27">
         <f>E26</f>
         <v>91.828309176174798</v>
@@ -5405,17 +5405,17 @@
         <f t="shared" si="22"/>
         <v>2.0128981508071853E-3</v>
       </c>
-      <c r="M27" s="4"/>
-      <c r="N27" s="4"/>
+      <c r="M27" s="5"/>
+      <c r="N27" s="5"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="5">
         <v>0.1115</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="5">
         <v>25.06</v>
       </c>
       <c r="D28">
@@ -5453,16 +5453,16 @@
         <f t="shared" ref="L28:L30" si="25">ABS(H28-K28)</f>
         <v>1.1916025071987413E-3</v>
       </c>
-      <c r="M28" s="4">
+      <c r="M28" s="5">
         <f>SUM(L28:L30)</f>
         <v>6.8379533125184633E-2</v>
       </c>
-      <c r="N28" s="4"/>
+      <c r="N28" s="5"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
       <c r="D29">
         <f>E28</f>
         <v>19.2292181061114</v>
@@ -5498,13 +5498,13 @@
         <f t="shared" si="25"/>
         <v>4.4913813788436396E-2</v>
       </c>
-      <c r="M29" s="4"/>
-      <c r="N29" s="4"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
       <c r="D30">
         <f>E29</f>
         <v>75.007571946818402</v>
@@ -5540,33 +5540,14 @@
         <f t="shared" si="25"/>
         <v>2.2274116829549495E-2</v>
       </c>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="N1:W1"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="A28:A30"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="M28:N30"/>
+    <mergeCell ref="M11:N12"/>
+    <mergeCell ref="M13:N15"/>
     <mergeCell ref="L10:N10"/>
     <mergeCell ref="A9:N9"/>
     <mergeCell ref="M16:N18"/>
@@ -5583,9 +5564,28 @@
     <mergeCell ref="M19:N21"/>
     <mergeCell ref="M22:N24"/>
     <mergeCell ref="M25:N27"/>
-    <mergeCell ref="M28:N30"/>
-    <mergeCell ref="M11:N12"/>
-    <mergeCell ref="M13:N15"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="N1:W1"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="R2:S2"/>
   </mergeCells>
   <conditionalFormatting sqref="M11:N30">
     <cfRule type="colorScale" priority="1">

</xml_diff>